<commit_message>
JT-263 Fix typos in template and sample Excel files
</commit_message>
<xml_diff>
--- a/resources/Samples/full_dataset_sample.xlsx
+++ b/resources/Samples/full_dataset_sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C1E286-76C3-4DA6-95E6-E4018ACF2682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4524FDDE-2C3D-482E-BE5B-27028DD4B920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8580" yWindow="10830" windowWidth="33090" windowHeight="19545" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="4200" yWindow="4200" windowWidth="43200" windowHeight="23445" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="226">
   <si>
     <t>IssueType</t>
   </si>
@@ -240,9 +240,6 @@
   </si>
   <si>
     <t>Fix Version</t>
-  </si>
-  <si>
-    <t>Asssignee.Name</t>
   </si>
   <si>
     <t>Assignee.ID</t>
@@ -1363,9 +1360,6 @@
   </cellStyles>
   <dxfs count="58">
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
       </fill>
@@ -1508,9 +1502,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1605,6 +1596,12 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="top"/>
@@ -1708,45 +1705,45 @@
     <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="49"/>
     <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="48"/>
     <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="47"/>
-    <tableColumn id="31" xr3:uid="{DA0D5F8E-BF5F-462C-B819-B0CE3CF6918C}" name="CF Number" dataDxfId="17"/>
-    <tableColumn id="32" xr3:uid="{49F51846-B44C-482E-BB5B-806FFDC85264}" name="CF Plain Text" dataDxfId="0"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="45"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="44"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="43"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="42">
+    <tableColumn id="31" xr3:uid="{DA0D5F8E-BF5F-462C-B819-B0CE3CF6918C}" name="CF Number" dataDxfId="46"/>
+    <tableColumn id="32" xr3:uid="{49F51846-B44C-482E-BB5B-806FFDC85264}" name="CF Plain Text" dataDxfId="45"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="43"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="41"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="40">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="41"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="40"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="31"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="30"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="29"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="28"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="27">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="39"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="38"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="36"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="35"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="34"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="33"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="32"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="31"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="30"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="29"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="28"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="27"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="26"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="25">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="26">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="24">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="25">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="24">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="23">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="21">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="22">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="20">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1762,7 +1759,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="21">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="19">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1772,7 +1769,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="20"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1825,7 +1822,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1835,7 +1832,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}" name="CfgAssignees" displayName="CfgAssignees" ref="A3:B8" totalsRowShown="0">
   <autoFilter ref="A3:B8" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7F7B4E10-E51C-443F-875D-3E6A9FD9994C}" name="Asssignee.Name"/>
+    <tableColumn id="1" xr3:uid="{7F7B4E10-E51C-443F-875D-3E6A9FD9994C}" name="Assignee.Name"/>
     <tableColumn id="2" xr3:uid="{3A4C6F03-89A9-4E38-8288-00D055D51CD3}" name="Assignee.ID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1859,7 +1856,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2258,10 +2255,10 @@
         <v>8</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>9</v>
@@ -2270,7 +2267,7 @@
         <v>10</v>
       </c>
       <c r="N1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O1" s="3" t="s">
         <v>11</v>
@@ -2364,7 +2361,7 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
@@ -2439,36 +2436,36 @@
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3">
         <v>1</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M3" s="3">
         <v>1</v>
@@ -2548,34 +2545,34 @@
         <v>38</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F4" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3">
         <v>1</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M4" s="3">
         <v>2</v>
@@ -2657,34 +2654,34 @@
         <v>47</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F5" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3">
         <v>1</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M5" s="3">
         <v>3</v>
@@ -2763,37 +2760,37 @@
     </row>
     <row r="6" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F6" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3">
         <v>1</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M6" s="3">
         <v>4</v>
@@ -2875,34 +2872,34 @@
         <v>42</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F7" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3">
         <v>1</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M7" s="3">
         <v>5</v>
@@ -2984,34 +2981,34 @@
         <v>48</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F8" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3">
         <v>1</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M8" s="3">
         <v>6</v>
@@ -3096,28 +3093,28 @@
         <v>37</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F9" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3">
         <v>1</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L9" s="3">
         <v>1.1000000000000001</v>
@@ -3199,37 +3196,37 @@
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F10" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3">
         <v>1</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M10" s="3">
         <v>8</v>
@@ -3311,34 +3308,34 @@
         <v>38</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F11" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3">
         <v>1</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M11" s="3">
         <v>9</v>
@@ -3420,34 +3417,34 @@
         <v>47</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F12" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3">
         <v>1</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M12" s="3">
         <v>10</v>
@@ -3529,34 +3526,34 @@
         <v>42</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F13" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3">
         <v>1</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M13" s="3">
         <v>11</v>
@@ -3635,37 +3632,37 @@
     </row>
     <row r="14" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F14" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3">
         <v>1</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M14" s="3">
         <v>12</v>
@@ -3747,34 +3744,34 @@
         <v>38</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F15" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3">
         <v>1</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M15" s="3">
         <v>13</v>
@@ -3856,34 +3853,34 @@
         <v>48</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F16" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="3">
         <v>1</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M16" s="3">
         <v>14</v>
@@ -3965,34 +3962,34 @@
         <v>49</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F17" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I17" s="3"/>
       <c r="J17" s="3">
         <v>1</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M17" s="3">
         <v>15</v>
@@ -4074,34 +4071,34 @@
         <v>38</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F18" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I18" s="3"/>
       <c r="J18" s="3">
         <v>1</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M18" s="3">
         <v>16</v>
@@ -4180,37 +4177,37 @@
     </row>
     <row r="19" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F19" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3">
         <v>1</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M19" s="3">
         <v>17</v>
@@ -4290,34 +4287,34 @@
         <v>38</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F20" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3">
         <v>1</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M20" s="3">
         <v>18</v>
@@ -4399,34 +4396,34 @@
         <v>47</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F21" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3">
         <v>1</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M21" s="3">
         <v>19</v>
@@ -4505,37 +4502,37 @@
     </row>
     <row r="22" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F22" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I22" s="3"/>
       <c r="J22" s="3">
         <v>1</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M22" s="3">
         <v>20</v>
@@ -4617,34 +4614,34 @@
         <v>42</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F23" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I23" s="3"/>
       <c r="J23" s="3">
         <v>1</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M23" s="3">
         <v>21</v>
@@ -4726,34 +4723,34 @@
         <v>48</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F24" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I24" s="3"/>
       <c r="J24" s="3">
         <v>1</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M24" s="3">
         <v>22</v>
@@ -4835,34 +4832,34 @@
         <v>49</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F25" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I25" s="3"/>
       <c r="J25" s="3">
         <v>1</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M25" s="3">
         <v>23</v>
@@ -4941,37 +4938,37 @@
     </row>
     <row r="26" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F26" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I26" s="3"/>
       <c r="J26" s="3">
         <v>1</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M26" s="3">
         <v>24</v>
@@ -5053,34 +5050,34 @@
         <v>38</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F27" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3">
         <v>1</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M27" s="3">
         <v>25</v>
@@ -5162,34 +5159,34 @@
         <v>47</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F28" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I28" s="3"/>
       <c r="J28" s="3">
         <v>1</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M28" s="3">
         <v>26</v>
@@ -5271,34 +5268,34 @@
         <v>42</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F29" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3">
         <v>1</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M29" s="3">
         <v>27</v>
@@ -5377,37 +5374,37 @@
     </row>
     <row r="30" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F30" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3">
         <v>1</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M30" s="3">
         <v>28</v>
@@ -5489,34 +5486,34 @@
         <v>38</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F31" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3">
         <v>1</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M31" s="3">
         <v>29</v>
@@ -5598,34 +5595,34 @@
         <v>48</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F32" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I32" s="3"/>
       <c r="J32" s="3">
         <v>1</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M32" s="3">
         <v>30</v>
@@ -5707,34 +5704,34 @@
         <v>49</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F33" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I33" s="3"/>
       <c r="J33" s="3">
         <v>1</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M33" s="3">
         <v>31</v>
@@ -5816,34 +5813,34 @@
         <v>38</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F34" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I34" s="3"/>
       <c r="J34" s="3">
         <v>1</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M34" s="3">
         <v>32</v>
@@ -5922,37 +5919,37 @@
     </row>
     <row r="35" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F35" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3">
         <v>1</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M35" s="3">
         <v>33</v>
@@ -6034,34 +6031,34 @@
         <v>38</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F36" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I36" s="3"/>
       <c r="J36" s="3">
         <v>1</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M36" s="3">
         <v>34</v>
@@ -6143,34 +6140,34 @@
         <v>47</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F37" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="3">
         <v>1</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M37" s="3">
         <v>35</v>
@@ -6252,34 +6249,34 @@
         <v>42</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F38" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3">
         <v>1</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M38" s="3">
         <v>36</v>
@@ -6361,34 +6358,34 @@
         <v>48</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F39" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3">
         <v>1</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M39" s="3">
         <v>37</v>
@@ -6470,34 +6467,34 @@
         <v>49</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F40" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I40" s="3"/>
       <c r="J40" s="3">
         <v>1</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M40" s="3">
         <v>38</v>
@@ -6576,37 +6573,37 @@
     </row>
     <row r="41" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F41" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I41" s="3"/>
       <c r="J41" s="3">
         <v>1</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M41" s="3">
         <v>39</v>
@@ -6688,34 +6685,34 @@
         <v>38</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F42" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I42" s="3"/>
       <c r="J42" s="3">
         <v>1</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M42" s="3">
         <v>40</v>
@@ -6799,64 +6796,64 @@
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
   <conditionalFormatting sqref="A2:A42 C2:C42">
-    <cfRule type="containsText" dxfId="16" priority="429" operator="containsText" text="blocker">
+    <cfRule type="containsText" dxfId="15" priority="429" operator="containsText" text="blocker">
       <formula>NOT(ISERROR(SEARCH("blocker",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="430" operator="containsText" text="critical">
+    <cfRule type="containsText" dxfId="14" priority="430" operator="containsText" text="critical">
       <formula>NOT(ISERROR(SEARCH("critical",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="431" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="13" priority="431" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="432" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="12" priority="432" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A42">
-    <cfRule type="containsBlanks" dxfId="12" priority="493">
+    <cfRule type="containsBlanks" dxfId="11" priority="493">
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:AL42">
-    <cfRule type="expression" dxfId="11" priority="409" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="409" stopIfTrue="1">
       <formula>$B2=cfg_type_comment</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="410">
+    <cfRule type="expression" dxfId="9" priority="410">
       <formula>$B2=cfg_type_skip</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="411">
+    <cfRule type="expression" dxfId="8" priority="411">
       <formula>$B2=cfg_type_note</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B42">
-    <cfRule type="containsText" dxfId="8" priority="413" operator="containsText" text="epic">
+    <cfRule type="containsText" dxfId="7" priority="413" operator="containsText" text="epic">
       <formula>NOT(ISERROR(SEARCH("epic",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="427" operator="containsText" text="story">
+    <cfRule type="containsText" dxfId="6" priority="427" operator="containsText" text="story">
       <formula>NOT(ISERROR(SEARCH("story",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="433" operator="containsText" text="task">
+    <cfRule type="containsText" dxfId="5" priority="433" operator="containsText" text="task">
       <formula>NOT(ISERROR(SEARCH("task",B2)))</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="5" priority="492">
+    <cfRule type="containsBlanks" dxfId="4" priority="492">
       <formula>LEN(TRIM(B2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:AL42">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$B2="Epic"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$B2="Story"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C42">
-    <cfRule type="containsBlanks" dxfId="2" priority="494">
+    <cfRule type="containsBlanks" dxfId="1" priority="494">
       <formula>LEN(TRIM(C2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:N42">
-    <cfRule type="containsBlanks" dxfId="1" priority="412">
+    <cfRule type="containsBlanks" dxfId="0" priority="412">
       <formula>LEN(TRIM(M2))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6884,7 +6881,7 @@
       <formula1>INDIRECT("CfgComponents[Component.Name]")</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="warning" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G42" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
-      <formula1>INDIRECT("CfgAssignees[Asssignee.Name]")</formula1>
+      <formula1>INDIRECT("CfgAssignees[Assignee.Name]")</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I42" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
       <formula1>INDIRECT("CfgSprints[Sprint.Name]")</formula1>
@@ -6958,11 +6955,11 @@
   <sheetData>
     <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B1" s="12"/>
       <c r="D1" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E1" s="12"/>
       <c r="G1" s="6" t="s">
@@ -6975,55 +6972,55 @@
         <v>51</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>52</v>
       </c>
       <c r="Q1" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R1" s="12"/>
       <c r="S1" s="12"/>
       <c r="U1" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="V1" s="12"/>
       <c r="W1" s="12"/>
       <c r="X1" s="12"/>
       <c r="Z1" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="7"/>
       <c r="D2" s="13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E2" s="13"/>
       <c r="F2" s="7"/>
       <c r="G2" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L2" s="13"/>
       <c r="M2" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="13"/>
@@ -7036,37 +7033,37 @@
       <c r="X2" s="7"/>
       <c r="Y2" s="7"/>
       <c r="Z2" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AA2" s="9"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
         <v>57</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>58</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>59</v>
       </c>
-      <c r="E3" t="s">
-        <v>60</v>
-      </c>
       <c r="G3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="Q3" t="s">
         <v>53</v>
@@ -7075,36 +7072,36 @@
         <v>54</v>
       </c>
       <c r="S3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="U3" t="s">
         <v>53</v>
       </c>
       <c r="V3" t="s">
+        <v>210</v>
+      </c>
+      <c r="W3" t="s">
         <v>211</v>
       </c>
-      <c r="W3" t="s">
+      <c r="X3" t="s">
         <v>212</v>
       </c>
-      <c r="X3" t="s">
-        <v>213</v>
-      </c>
       <c r="Z3" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -7119,17 +7116,17 @@
         <v>50</v>
       </c>
       <c r="R4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="S4" s="7"/>
       <c r="U4" t="s">
+        <v>213</v>
+      </c>
+      <c r="V4" t="s">
         <v>214</v>
       </c>
-      <c r="V4" t="s">
+      <c r="W4" t="s">
         <v>215</v>
-      </c>
-      <c r="W4" t="s">
-        <v>216</v>
       </c>
       <c r="Z4" t="str" cm="1">
         <f t="array" aca="1" ref="Z4:Z13" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
@@ -7138,16 +7135,16 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K5" t="s">
         <v>37</v>
@@ -7162,19 +7159,19 @@
         <v>46</v>
       </c>
       <c r="R5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="U5" t="s">
+        <v>216</v>
+      </c>
+      <c r="V5" t="s">
         <v>217</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>218</v>
-      </c>
-      <c r="W5" t="s">
-        <v>219</v>
       </c>
       <c r="Z5" t="str">
         <f ca="1"/>
@@ -7183,16 +7180,16 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K6" t="s">
         <v>40</v>
@@ -7201,25 +7198,25 @@
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Q6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="U6" t="s">
+        <v>219</v>
+      </c>
+      <c r="V6" t="s">
         <v>220</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>221</v>
-      </c>
-      <c r="W6" t="s">
-        <v>222</v>
       </c>
       <c r="Z6" t="str">
         <f ca="1"/>
@@ -7228,15 +7225,15 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="I7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K7" t="s">
         <v>41</v>
@@ -7248,20 +7245,20 @@
         <v>42</v>
       </c>
       <c r="Q7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="R7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="S7" s="7"/>
       <c r="U7" t="s">
+        <v>222</v>
+      </c>
+      <c r="V7" t="s">
         <v>223</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>224</v>
-      </c>
-      <c r="W7" t="s">
-        <v>225</v>
       </c>
       <c r="Z7" t="str">
         <f ca="1"/>
@@ -7270,24 +7267,24 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" t="s">
         <v>109</v>
-      </c>
-      <c r="B8" t="s">
-        <v>110</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="I8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>48</v>
       </c>
       <c r="Q8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
@@ -7302,19 +7299,19 @@
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="I9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>49</v>
       </c>
       <c r="Q9" t="s">
+        <v>203</v>
+      </c>
+      <c r="R9" t="s">
         <v>204</v>
-      </c>
-      <c r="R9" t="s">
-        <v>205</v>
       </c>
       <c r="S9" s="7"/>
       <c r="Z9" t="str">
@@ -7326,7 +7323,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="I10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Z10" t="str">
         <f ca="1"/>
@@ -7337,7 +7334,7 @@
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="I11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Z11" t="str">
         <f ca="1"/>
@@ -7424,6 +7421,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -7652,27 +7669,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7689,23 +7705,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-71 Add support for Compass components in configuration
- Introduced `jira.components_source` option to specify the use of Compass components in Jira Software spaces.
- Updated documentation to include examples for JSON and Excel configurations.

related: JT-87
</commit_message>
<xml_diff>
--- a/resources/Samples/full_dataset_sample.xlsx
+++ b/resources/Samples/full_dataset_sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4524FDDE-2C3D-482E-BE5B-27028DD4B920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E3904B-91CA-4C4A-98F0-58D7867110F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="4200" windowWidth="43200" windowHeight="23445" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="4245" yWindow="4245" windowWidth="31710" windowHeight="20325" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="228">
   <si>
     <t>IssueType</t>
   </si>
@@ -747,6 +747,12 @@
   </si>
   <si>
     <t>abc</t>
+  </si>
+  <si>
+    <t>jira.components_source</t>
+  </si>
+  <si>
+    <t>jira</t>
   </si>
 </sst>
 </file>
@@ -1851,8 +1857,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S9" totalsRowShown="0">
-  <autoFilter ref="Q3:S9" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S10" totalsRowShown="0">
+  <autoFilter ref="Q3:S10" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
@@ -7325,6 +7331,13 @@
       <c r="I10" t="s">
         <v>97</v>
       </c>
+      <c r="Q10" t="s">
+        <v>226</v>
+      </c>
+      <c r="R10" t="s">
+        <v>227</v>
+      </c>
+      <c r="S10" s="7"/>
       <c r="Z10" t="str">
         <f ca="1"/>
         <v>Comment</v>
@@ -7421,26 +7434,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -7669,26 +7662,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7705,4 +7699,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-143 feat: update config_sample.json with new config version 8. Update full_dataset_sample.xlsx for compatibility.
</commit_message>
<xml_diff>
--- a/resources/Samples/full_dataset_sample.xlsx
+++ b/resources/Samples/full_dataset_sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD5FD0F-7840-4E78-8412-F4D2762CDDC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{489CD560-7F1F-41CD-BBC2-BBB3D5B1596E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4380" yWindow="2970" windowWidth="29685" windowHeight="23445" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="31785" activeTab="5" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -24,9 +24,9 @@
     <sheet name="_ImportReport" sheetId="8" state="hidden" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="cfg_labels_ft_label">'Config - Basic'!$B$6</definedName>
-    <definedName name="cfg_labels_ft_name">'Config - Basic'!$B$6</definedName>
-    <definedName name="cfg_labels_imported">'Config - Basic'!$B$5</definedName>
+    <definedName name="cfg_labels_ft_label">'Config - Basic'!#REF!</definedName>
+    <definedName name="cfg_labels_ft_name">'Config - Basic'!#REF!</definedName>
+    <definedName name="cfg_labels_imported">'Config - Basic'!#REF!</definedName>
     <definedName name="cfg_projectKey">'Config - Basic'!$B$4</definedName>
     <definedName name="cfg_type_comment">'Config - Factory'!$I$4</definedName>
     <definedName name="cfg_type_note">'Config - Factory'!$I$6</definedName>
@@ -36,7 +36,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId10"/>
+    <pivotCache cacheId="0" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -246,7 +246,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="290">
   <si>
     <t>IssueType</t>
   </si>
@@ -383,9 +383,6 @@
     <t>WorkItem</t>
   </si>
   <si>
-    <t>Feature Pod Label</t>
-  </si>
-  <si>
     <t>Highest</t>
   </si>
   <si>
@@ -1107,6 +1104,18 @@
   </si>
   <si>
     <t>4h</t>
+  </si>
+  <si>
+    <t>Team 1</t>
+  </si>
+  <si>
+    <t>Team 2</t>
+  </si>
+  <si>
+    <t>2342342340:09876543212345678901</t>
+  </si>
+  <si>
+    <t>2342342340:0987654321234567890456</t>
   </si>
 </sst>
 </file>
@@ -1888,6 +1897,9 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2034,9 +2046,6 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2293,7 +2302,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9326BD75-A09D-4578-BB55-882D1F75C66E}" name="PT_Issues" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9326BD75-A09D-4578-BB55-882D1F75C66E}" name="PT_Issues" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="36">
     <pivotField showAll="0"/>
@@ -2401,7 +2410,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A931C4D6-0F40-4FC0-8FE0-7829E37288EB}" name="PT_Assignees" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A931C4D6-0F40-4FC0-8FE0-7829E37288EB}" name="PT_Assignees" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="D5:E10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="36">
     <pivotField showAll="0"/>
@@ -2546,57 +2555,57 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ42" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ42" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="A1:AJ42" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="53"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="51"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="50"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="49">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="50">
       <calculatedColumnFormula>'Config - Mappings'!$J$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="47"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="46"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="45"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="44"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="43"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="42"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="41">
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="49"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="48"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="47"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="45"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="44"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="43"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="42">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="40"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="39"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="38"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="37"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="36"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="35"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="34"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="33"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="32"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="31"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="30"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="29"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="28"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="27"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="26">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="41"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="40"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="39"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="38"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="37"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="36"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="35"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="34"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="33"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="32"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="31"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="30"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="29"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="28"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="27">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], 'Config - Mappings'!$G$4:$H$8, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="25">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="26">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="24">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="25">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Work Group", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="23">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="24">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], 'Config - Mappings'!$A$4:$B$26, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="22">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgBasic[Name], CfgBasic[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="21">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="22">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -2612,7 +2621,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="20">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="21">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -2622,7 +2631,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="19"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2632,15 +2641,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="L22:L28" totalsRowShown="0">
   <autoFilter ref="L22:L28" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{DE352608-207B-4EFC-9BD3-2BD6976D373F}" name="CfgTeams" displayName="CfgTeams" ref="D3:E9" totalsRowShown="0">
-  <autoFilter ref="D3:E9" xr:uid="{DE352608-207B-4EFC-9BD3-2BD6976D373F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{DE352608-207B-4EFC-9BD3-2BD6976D373F}" name="CfgTeams" displayName="CfgTeams" ref="D3:E6" totalsRowShown="0">
+  <autoFilter ref="D3:E6" xr:uid="{DE352608-207B-4EFC-9BD3-2BD6976D373F}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{59E7B951-2640-4BEF-926D-11574E54F447}" name="Team.Name"/>
     <tableColumn id="2" xr3:uid="{1C40E406-7D3C-45A3-AAA3-B5BBB7E9C3AA}" name="Team.ID"/>
@@ -2719,12 +2728,12 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgBasic" displayName="CfgBasic" ref="A3:C7" totalsRowShown="0">
-  <autoFilter ref="A3:C7" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgBasic" displayName="CfgBasic" ref="A3:C5" totalsRowShown="0">
+  <autoFilter ref="A3:C5" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2736,7 +2745,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{19232286-858A-4316-B524-2259E904D535}" name="Name"/>
     <tableColumn id="2" xr3:uid="{E6137B31-22A5-4579-8A81-0FBB4015A668}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{03DA91C8-48E1-4BFC-B993-8C1071BAA534}" name="Note" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{03DA91C8-48E1-4BFC-B993-8C1071BAA534}" name="Note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3182,7 +3191,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -3267,7 +3276,7 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -3347,28 +3356,28 @@
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K3" s="3">
         <v>1</v>
@@ -3383,13 +3392,13 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="S3" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="T3" s="3" t="s">
         <v>161</v>
-      </c>
-      <c r="T3" s="3" t="s">
-        <v>162</v>
       </c>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
@@ -3454,27 +3463,27 @@
         <v>37</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K4" s="3">
         <v>2</v>
@@ -3553,30 +3562,30 @@
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K5" s="3">
         <v>3</v>
@@ -3655,30 +3664,30 @@
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="K6" s="3">
         <v>4</v>
@@ -3757,30 +3766,30 @@
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="K7" s="3">
         <v>5</v>
@@ -3859,30 +3868,30 @@
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K8" s="3">
         <v>6</v>
@@ -3961,30 +3970,30 @@
     </row>
     <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K9" s="3">
         <v>7</v>
@@ -4063,30 +4072,30 @@
     </row>
     <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K10" s="3">
         <v>8</v>
@@ -4168,27 +4177,27 @@
         <v>37</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K11" s="3">
         <v>9</v>
@@ -4267,30 +4276,30 @@
     </row>
     <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K12" s="3">
         <v>10</v>
@@ -4369,30 +4378,30 @@
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="K13" s="3">
         <v>11</v>
@@ -4471,30 +4480,30 @@
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K14" s="3">
         <v>12</v>
@@ -4576,27 +4585,27 @@
         <v>37</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K15" s="3">
         <v>13</v>
@@ -4675,30 +4684,30 @@
     </row>
     <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K16" s="3">
         <v>14</v>
@@ -4777,30 +4786,30 @@
     </row>
     <row r="17" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I17" s="3"/>
       <c r="J17" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K17" s="3">
         <v>15</v>
@@ -4882,27 +4891,27 @@
         <v>37</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I18" s="3"/>
       <c r="J18" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K18" s="3">
         <v>16</v>
@@ -4981,30 +4990,30 @@
     </row>
     <row r="19" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K19" s="3">
         <v>17</v>
@@ -5084,27 +5093,27 @@
         <v>37</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K20" s="3">
         <v>18</v>
@@ -5183,30 +5192,30 @@
     </row>
     <row r="21" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K21" s="3">
         <v>19</v>
@@ -5285,30 +5294,30 @@
     </row>
     <row r="22" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I22" s="3"/>
       <c r="J22" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K22" s="3">
         <v>20</v>
@@ -5387,30 +5396,30 @@
     </row>
     <row r="23" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I23" s="3"/>
       <c r="J23" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="K23" s="3">
         <v>21</v>
@@ -5489,30 +5498,30 @@
     </row>
     <row r="24" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I24" s="3"/>
       <c r="J24" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K24" s="3">
         <v>22</v>
@@ -5591,30 +5600,30 @@
     </row>
     <row r="25" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I25" s="3"/>
       <c r="J25" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K25" s="3">
         <v>23</v>
@@ -5693,30 +5702,30 @@
     </row>
     <row r="26" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I26" s="3"/>
       <c r="J26" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K26" s="3">
         <v>24</v>
@@ -5798,27 +5807,27 @@
         <v>37</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K27" s="3">
         <v>25</v>
@@ -5897,30 +5906,30 @@
     </row>
     <row r="28" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I28" s="3"/>
       <c r="J28" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K28" s="3">
         <v>26</v>
@@ -5999,30 +6008,30 @@
     </row>
     <row r="29" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="K29" s="3">
         <v>27</v>
@@ -6101,30 +6110,30 @@
     </row>
     <row r="30" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K30" s="3">
         <v>28</v>
@@ -6206,27 +6215,27 @@
         <v>37</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K31" s="3">
         <v>29</v>
@@ -6305,30 +6314,30 @@
     </row>
     <row r="32" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I32" s="3"/>
       <c r="J32" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K32" s="3">
         <v>30</v>
@@ -6407,30 +6416,30 @@
     </row>
     <row r="33" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I33" s="3"/>
       <c r="J33" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K33" s="3">
         <v>31</v>
@@ -6512,27 +6521,27 @@
         <v>37</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I34" s="3"/>
       <c r="J34" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K34" s="3">
         <v>32</v>
@@ -6611,30 +6620,30 @@
     </row>
     <row r="35" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K35" s="3">
         <v>33</v>
@@ -6716,27 +6725,27 @@
         <v>37</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I36" s="3"/>
       <c r="J36" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K36" s="3">
         <v>34</v>
@@ -6815,30 +6824,30 @@
     </row>
     <row r="37" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K37" s="3">
         <v>35</v>
@@ -6917,30 +6926,30 @@
     </row>
     <row r="38" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K38" s="3">
         <v>36</v>
@@ -7019,30 +7028,30 @@
     </row>
     <row r="39" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K39" s="3">
         <v>37</v>
@@ -7121,30 +7130,30 @@
     </row>
     <row r="40" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I40" s="3"/>
       <c r="J40" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K40" s="3">
         <v>38</v>
@@ -7223,30 +7232,30 @@
     </row>
     <row r="41" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I41" s="3"/>
       <c r="J41" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K41" s="3">
         <v>39</v>
@@ -7328,27 +7337,27 @@
         <v>37</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I42" s="3"/>
       <c r="J42" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K42" s="3">
         <v>40</v>
@@ -7565,7 +7574,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -7573,34 +7582,34 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -7614,13 +7623,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -7642,13 +7651,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -7656,13 +7665,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E10">
         <v>2</v>
@@ -7678,7 +7687,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -7704,14 +7713,14 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B2" s="17"/>
       <c r="C2" t="str">
@@ -7721,47 +7730,47 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -7770,19 +7779,19 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B9" s="17">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" s="17"/>
       <c r="C10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -7790,13 +7799,13 @@
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B12" s="17"/>
       <c r="C12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -7816,17 +7825,17 @@
     </row>
     <row r="19" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A19" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C21" t="s">
         <v>4</v>
@@ -7834,13 +7843,13 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>104</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -7849,21 +7858,21 @@
         <v>CfgBasic</v>
       </c>
       <c r="B23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>106</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -7872,10 +7881,10 @@
         <v>CfgAssignees</v>
       </c>
       <c r="B25" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -7884,10 +7893,10 @@
         <v>CfgSprints</v>
       </c>
       <c r="B26" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -7896,10 +7905,10 @@
         <v>CfgFixVersions</v>
       </c>
       <c r="B27" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -7908,10 +7917,10 @@
         <v>CfgIssueTypes</v>
       </c>
       <c r="B28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -7920,10 +7929,10 @@
         <v>CfgComponents</v>
       </c>
       <c r="B29" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C29" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -7932,21 +7941,21 @@
         <v>CfgPriorities</v>
       </c>
       <c r="B30" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C30" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -7955,10 +7964,10 @@
         <v>CfgAdvanced</v>
       </c>
       <c r="B32" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C32" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -7967,21 +7976,21 @@
         <v>CfgCustomFields</v>
       </c>
       <c r="B33" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C33" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -7990,10 +7999,10 @@
         <v>CfgSettings</v>
       </c>
       <c r="B35" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C35" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -8002,21 +8011,21 @@
         <v>CfgAutofieldValues</v>
       </c>
       <c r="B36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C36" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C37" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -8025,15 +8034,15 @@
         <v>cfg_type_note</v>
       </c>
       <c r="B38" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C38" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C45" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -8060,7 +8069,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
@@ -8073,43 +8082,43 @@
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="E1" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F1" s="18"/>
       <c r="G1" s="18"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="8"/>
       <c r="E2" s="19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F2" s="19"/>
       <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
         <v>51</v>
-      </c>
-      <c r="B3" t="s">
-        <v>52</v>
       </c>
       <c r="C3" t="s">
         <v>33</v>
       </c>
       <c r="E3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" t="s">
         <v>51</v>
-      </c>
-      <c r="F3" t="s">
-        <v>52</v>
       </c>
       <c r="G3" t="s">
         <v>33</v>
@@ -8117,63 +8126,41 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
         <v>39</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="E5" t="s">
+        <v>176</v>
+      </c>
+      <c r="F5" t="s">
+        <v>79</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="E5" t="s">
-        <v>177</v>
-      </c>
-      <c r="F5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -8182,10 +8169,13 @@
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="E2:G2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{9CF84CAA-87E5-4B56-A1A8-8714F7942F16}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8211,42 +8201,42 @@
   <sheetData>
     <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B1" s="18"/>
       <c r="D1" s="18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E1" s="18"/>
       <c r="G1" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H1" s="18"/>
       <c r="J1" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E2" s="19"/>
       <c r="G2" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H2" s="19"/>
       <c r="J2" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -8254,45 +8244,45 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G3" t="s">
         <v>55</v>
       </c>
-      <c r="D3" t="s">
-        <v>172</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M3" t="s">
         <v>173</v>
-      </c>
-      <c r="G3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J3" t="s">
-        <v>61</v>
-      </c>
-      <c r="L3" t="s">
-        <v>59</v>
-      </c>
-      <c r="M3" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D4" t="s">
-        <v>148</v>
+        <v>286</v>
       </c>
       <c r="E4" t="s">
-        <v>153</v>
+        <v>288</v>
       </c>
       <c r="J4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L4" t="s">
         <v>38</v>
@@ -8303,19 +8293,19 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D5" t="s">
-        <v>149</v>
+        <v>287</v>
       </c>
       <c r="E5" t="s">
-        <v>154</v>
+        <v>289</v>
       </c>
       <c r="J5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="L5" t="s">
         <v>36</v>
@@ -8326,21 +8316,15 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B6" t="s">
-        <v>155</v>
-      </c>
-      <c r="D6" t="s">
-        <v>150</v>
-      </c>
-      <c r="E6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="J6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L6" t="s">
         <v>40</v>
@@ -8351,16 +8335,10 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B7" t="s">
-        <v>156</v>
-      </c>
-      <c r="D7" t="s">
-        <v>151</v>
-      </c>
-      <c r="E7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -8373,21 +8351,15 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B8" t="s">
-        <v>157</v>
-      </c>
-      <c r="D8" t="s">
-        <v>152</v>
-      </c>
-      <c r="E8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="L8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M8">
         <v>4</v>
@@ -8397,7 +8369,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="L9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M9">
         <v>1</v>
@@ -8447,31 +8419,31 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="J20" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J21" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J23" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="L23" s="1" t="s">
         <v>37</v>
@@ -8479,62 +8451,62 @@
     </row>
     <row r="24" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J24" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J29" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J30" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="31" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J31" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="32" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J32" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -8576,12 +8548,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="E1" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F1" s="18"/>
       <c r="G1" s="18"/>
@@ -8598,47 +8570,47 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
         <v>51</v>
-      </c>
-      <c r="B3" t="s">
-        <v>52</v>
       </c>
       <c r="C3" t="s">
         <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" t="s">
         <v>95</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>96</v>
-      </c>
-      <c r="H3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" t="s">
         <v>85</v>
       </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
       <c r="C4" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" t="s">
         <v>87</v>
       </c>
-      <c r="B5" t="s">
-        <v>88</v>
-      </c>
       <c r="C5" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -8660,7 +8632,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
@@ -8672,46 +8644,46 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D1" s="18"/>
       <c r="F1" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G1" s="18"/>
       <c r="I1" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
         <v>51</v>
       </c>
-      <c r="D3" t="s">
-        <v>52</v>
-      </c>
       <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
         <v>51</v>
       </c>
-      <c r="G3" t="s">
-        <v>52</v>
-      </c>
       <c r="I3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -8720,7 +8692,7 @@
         <v>Story</v>
       </c>
       <c r="C4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D4">
         <v>8</v>
@@ -8735,7 +8707,7 @@
         <v>Task</v>
       </c>
       <c r="C5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D5" t="str" cm="1">
         <f t="array" aca="1" ref="D5" ca="1">"[" &amp; _xlfn.TEXTJOIN(",",TRUE,_xlfn.MAP(_xlfn._xlws.FILTER(INDIRECT("CfgIgnoreList[IgnoreList.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]")&lt;&gt;""),_xlfn.LAMBDA(_xlpm.x,"""" &amp; SUBSTITUTE(_xlpm.x,"""","""""") &amp; """"))) &amp; "]"</f>
@@ -8799,7 +8771,7 @@
         <v>WorkItem</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D13" s="18"/>
       <c r="E13" s="18"/>
@@ -8808,7 +8780,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C14" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
@@ -8817,7 +8789,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" t="str" cm="1">
-        <f t="array" aca="1" ref="C15:E21" ca="1">_xlfn.UNIQUE(
+        <f t="array" aca="1" ref="C15:E19" ca="1">_xlfn.UNIQUE(
     (
         _xlfn.VSTACK(
             INDIRECT("CfgBasic"),
@@ -8840,83 +8812,55 @@
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C16" t="str">
         <f ca="1"/>
-        <v>Creation Marker</v>
+        <v>jira.connection.site_address</v>
       </c>
       <c r="D16" t="str">
         <f ca="1"/>
-        <v>imported</v>
-      </c>
-      <c r="E16" t="str">
+        <v>https://deerhide.atlassian.net</v>
+      </c>
+      <c r="E16">
         <f ca="1"/>
-        <v>A label added to all imported task to flag them in Jira</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C17" t="str">
         <f ca="1"/>
-        <v>Feature Pod Label</v>
+        <v>app.import.auto_open_page</v>
       </c>
       <c r="D17" t="str">
         <f ca="1"/>
-        <v>pod_test</v>
+        <v>yes</v>
       </c>
       <c r="E17" t="str">
         <f ca="1"/>
-        <v>Appropirate label for the feature pod when relevant</v>
+        <v>Open the import page after processing the dataset?</v>
       </c>
     </row>
     <row r="18" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C18" t="str">
         <f ca="1"/>
-        <v>jira.connection.site_address</v>
+        <v>jira.components_source</v>
       </c>
       <c r="D18" t="str">
         <f ca="1"/>
-        <v>https://deerhide.atlassian.net</v>
-      </c>
-      <c r="E18">
+        <v>jira</v>
+      </c>
+      <c r="E18" t="str">
+        <f ca="1"/>
+        <v>Use Jira or Compass components</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C19">
         <f ca="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C19" t="str">
-        <f ca="1"/>
-        <v>app.import.auto_open_page</v>
-      </c>
-      <c r="D19" t="str">
-        <f ca="1"/>
-        <v>yes</v>
-      </c>
-      <c r="E19" t="str">
-        <f ca="1"/>
-        <v>Open the import page after processing the dataset?</v>
-      </c>
-    </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C20" t="str">
-        <f ca="1"/>
-        <v>jira.components_source</v>
-      </c>
-      <c r="D20" t="str">
-        <f ca="1"/>
-        <v>jira</v>
-      </c>
-      <c r="E20" t="str">
-        <f ca="1"/>
-        <v>Use Jira or Compass components</v>
-      </c>
-    </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C21">
+      <c r="D19">
         <f ca="1"/>
         <v>0</v>
       </c>
-      <c r="D21">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="E21" t="e">
+      <c r="E19" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
@@ -8962,14 +8906,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9202,21 +9144,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9241,9 +9182,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-51 Fix parent_link error in samples
</commit_message>
<xml_diff>
--- a/resources/Samples/full_dataset_sample.xlsx
+++ b/resources/Samples/full_dataset_sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{489CD560-7F1F-41CD-BBC2-BBB3D5B1596E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4354F84A-174A-4A63-950E-D865552F3BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="31785" activeTab="5" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="28365" yWindow="3015" windowWidth="26220" windowHeight="23385" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -1894,9 +1894,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -2046,6 +2043,9 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2555,57 +2555,57 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ42" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ42" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="A1:AJ42" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="54"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="53"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="52"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="51"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="50">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="51"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="49">
       <calculatedColumnFormula>'Config - Mappings'!$J$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="49"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="48"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="47"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="45"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="44"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="43"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="42">
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="46"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="45"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="44"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="42"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="41">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="41"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="40"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="31"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="30"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="29"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="28"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="27">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="40"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="39"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="38"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="37"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="36"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="35"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="34"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="33"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="32"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="31"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="30"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="29"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="28"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="27"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="26">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], 'Config - Mappings'!$G$4:$H$8, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="26">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="25">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="25">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="24">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Work Group", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="24">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], 'Config - Mappings'!$A$4:$B$26, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="23">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgBasic[Name], CfgBasic[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="22">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="21">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -2621,7 +2621,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="21">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="20">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -2631,7 +2631,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="20"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2641,7 +2641,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="L22:L28" totalsRowShown="0">
   <autoFilter ref="L22:L28" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2677,7 +2677,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{724752C0-2EB0-4307-9766-E95D142383BC}" name="Name"/>
     <tableColumn id="2" xr3:uid="{1B4D7FE1-60C9-4319-8B9F-E66C19764AEE}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{F0634D25-384E-480B-B675-9F8463C0D844}" name="Note" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{F0634D25-384E-480B-B675-9F8463C0D844}" name="Note" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2733,7 +2733,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2745,7 +2745,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{19232286-858A-4316-B524-2259E904D535}" name="Name"/>
     <tableColumn id="2" xr3:uid="{E6137B31-22A5-4579-8A81-0FBB4015A668}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{03DA91C8-48E1-4BFC-B993-8C1071BAA534}" name="Note" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{03DA91C8-48E1-4BFC-B993-8C1071BAA534}" name="Note" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4101,7 +4101,7 @@
         <v>8</v>
       </c>
       <c r="L10" s="3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M10" s="3"/>
       <c r="N10" s="3" t="str">
@@ -4203,7 +4203,7 @@
         <v>9</v>
       </c>
       <c r="L11" s="3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M11" s="3"/>
       <c r="N11" s="3" t="str">
@@ -4305,7 +4305,7 @@
         <v>10</v>
       </c>
       <c r="L12" s="3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M12" s="3"/>
       <c r="N12" s="3" t="str">
@@ -8906,12 +8906,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9144,20 +9146,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9182,12 +9185,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>